<commit_message>
Proyecto 2027: fuentes, parámetros y ejecución completa
Tomo 3 del Proyecto de Ley 2027, publicado el 2026-10-30, incorporado al
catálogo (sha256 9f847cb5) y procesado con todas las puertas en verde.

- fuentes.yml: entrada 2027 proyecto aceptada desde descubrir_fuentes.py.
- referencias_tomo3.yml: total 2.10 impreso en la p. 56 (12.542.221.590 €).
- transformacion.yml: IPC Canarias 2027 = 3,1 % (Tomo 4, cuadro 33) y límite
  de gasto no financiero 12.912.662,81 miles € (Acuerdo de 29-07-2026).
- externos_canarias.csv actualizado desde el INE (IPC 2026 con 9 meses).
- Crosswalks propuestos, salidas de análisis y CSV de la web regenerados.
  Un enlace nuevo pendiente de revisión: 432C (solo cambian abreviaturas).

Cargado en Supabase producción (presupuestos_can) el mismo día; coincide
fila a fila con DuckDB.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_analisis/salidas/entes/tablas_entes.xlsx
+++ b/4_analisis/salidas/entes/tablas_entes.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Peso de los entes en 2026</t>
+          <t>Peso de los entes en 2027</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Importe 2026 (M€)</t>
+          <t>Importe 2027 (M€)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -492,11 +492,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.833,5</t>
+          <t>5.245,6</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>86.18692167156483</v>
+        <v>86.29102126048345</v>
       </c>
     </row>
     <row r="6">
@@ -512,11 +512,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>351,4</t>
+          <t>351,5</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6.266143979567018</v>
+        <v>5.782250839705421</v>
       </c>
     </row>
     <row r="7">
@@ -532,11 +532,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>197,5</t>
+          <t>249,1</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3.520880965415776</v>
+        <v>4.096956126591778</v>
       </c>
     </row>
     <row r="8">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.145251118378188</v>
+        <v>1.056816423486834</v>
       </c>
     </row>
     <row r="9">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.086035761194509</v>
+        <v>1.001959247575999</v>
       </c>
     </row>
     <row r="10">
@@ -592,11 +592,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>41,1</t>
+          <t>48,5</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.7329187099546303</v>
+        <v>0.7979768980075765</v>
       </c>
     </row>
     <row r="11">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.2630145444186289</v>
+        <v>0.2426434890956023</v>
       </c>
     </row>
     <row r="12">
@@ -632,11 +632,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12,3</t>
+          <t>11,2</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.2184570165154288</v>
+        <v>0.1843170276458432</v>
       </c>
     </row>
     <row r="13">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.1940141179165712</v>
+        <v>0.1796726591332314</v>
       </c>
     </row>
     <row r="14">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.1393297340459139</v>
+        <v>0.1289255840321329</v>
       </c>
     </row>
     <row r="15">
@@ -692,11 +692,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6,5</t>
+          <t>7,0</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.115474976663312</v>
+        <v>0.1159234742651021</v>
       </c>
     </row>
     <row r="16">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.05889739289286249</v>
+        <v>0.05434442499333444</v>
       </c>
     </row>
     <row r="17">
@@ -732,11 +732,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2,4</t>
+          <t>2,5</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.04361413755247093</v>
+        <v>0.04037884687573817</v>
       </c>
     </row>
     <row r="18">
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.02592543028522558</v>
+        <v>0.02393492330646099</v>
       </c>
     </row>
     <row r="19">
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.003120443634634124</v>
+        <v>0.002878774801498472</v>
       </c>
     </row>
     <row r="21">
@@ -844,7 +844,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2027</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         <v>0.2577377899470507</v>
       </c>
       <c r="E5" t="n">
-        <v>0.221577460150063</v>
+        <v>0.1871958024473416</v>
       </c>
     </row>
     <row r="6">
@@ -883,7 +883,7 @@
         <v>2.797464786152288</v>
       </c>
       <c r="E6" t="n">
-        <v>2.274901017125168</v>
+        <v>2.099154517938572</v>
       </c>
     </row>
     <row r="7">
@@ -902,7 +902,7 @@
         <v>96.13010949725427</v>
       </c>
       <c r="E7" t="n">
-        <v>96.77060281277014</v>
+        <v>96.91567278160652</v>
       </c>
     </row>
     <row r="8">
@@ -917,7 +917,7 @@
         <v>0.8146879266463914</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.7329187099546303</v>
+        <v>0.7979768980075765</v>
       </c>
     </row>
     <row r="10">
@@ -1029,7 +1029,7 @@
         <v>2016</v>
       </c>
       <c r="C7" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1047,7 +1047,7 @@
         <v>2016</v>
       </c>
       <c r="C8" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>2022</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>

</xml_diff>